<commit_message>
finished keypad scanning code in monitor
keypad scanning plus some additional test and demonstration utilities.
</commit_message>
<xml_diff>
--- a/Documentation/Musical Tones.xlsx
+++ b/Documentation/Musical Tones.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/46a8e0c578cce4d5/Documents/Devel/MiniH8/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="8_{28299701-EF0E-4EA9-81EF-24F5FBAF51CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{025B2D4F-03DF-427D-A5B4-DA46AEFD00F6}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="8_{28299701-EF0E-4EA9-81EF-24F5FBAF51CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C1F1466-7ACE-4AFA-B911-82762F46827F}"/>
   <bookViews>
     <workbookView xWindow="10590" yWindow="255" windowWidth="21600" windowHeight="14535" xr2:uid="{A414EE4C-F510-43B6-8BCD-39260BAF1535}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="20">
   <si>
     <t>C</t>
   </si>
@@ -505,11 +505,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B96813B-94F5-45E1-A799-3EDA6A7EB35F}">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="4" width="9.140625" style="1"/>
-    <col min="6" max="7" width="9.140625" style="7"/>
+    <col min="2" max="4" width="9.140625" style="1" customWidth="1"/>
+    <col min="6" max="7" width="9.140625" style="7" customWidth="1"/>
     <col min="8" max="8" width="9.140625" style="8"/>
   </cols>
   <sheetData>
@@ -585,7 +585,7 @@
         <v>3.6077296635640912</v>
       </c>
       <c r="D3" s="1">
-        <f t="shared" ref="D3:D25" si="3">C3/2</f>
+        <f t="shared" ref="D1:D49" si="3">C3/2</f>
         <v>1.8038648317820456</v>
       </c>
       <c r="E3">
@@ -597,7 +597,7 @@
         <v>277.18263097687196</v>
       </c>
       <c r="G3" s="7">
-        <f t="shared" ref="G3:G25" si="5">F3/10</f>
+        <f t="shared" ref="G1:G49" si="5">F3/10</f>
         <v>27.718263097687196</v>
       </c>
       <c r="H3" s="8">
@@ -885,7 +885,7 @@
         <v>1.0725844462291971</v>
       </c>
       <c r="E12">
-        <f t="shared" ref="E12:E25" si="7">ROUND(D12*1000/9,0)</f>
+        <f t="shared" ref="E12:E49" si="7">ROUND(D12*1000/9,0)</f>
         <v>119</v>
       </c>
       <c r="F12" s="7">
@@ -976,7 +976,7 @@
         <v>554.36526195374427</v>
       </c>
       <c r="C15" s="1">
-        <f t="shared" ref="C15:C25" si="9">1/B15*1000</f>
+        <f t="shared" ref="C15:C49" si="9">1/B15*1000</f>
         <v>1.8038648317820445</v>
       </c>
       <c r="D15" s="1">
@@ -1328,6 +1328,798 @@
       <c r="H25" s="8">
         <f t="shared" si="6"/>
         <v>49.388330125612427</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B26" s="1">
+        <f t="shared" ref="B26" si="10">B25*POWER(2,1/12)</f>
+        <v>1046.5022612023949</v>
+      </c>
+      <c r="C26" s="1">
+        <f t="shared" si="9"/>
+        <v>0.95556410824285709</v>
+      </c>
+      <c r="D26" s="1">
+        <f t="shared" si="3"/>
+        <v>0.47778205412142855</v>
+      </c>
+      <c r="E26">
+        <f t="shared" si="7"/>
+        <v>53</v>
+      </c>
+      <c r="F26" s="7">
+        <f t="shared" ref="F26" si="11">1000/C26</f>
+        <v>1046.5022612023949</v>
+      </c>
+      <c r="G26" s="7">
+        <f t="shared" si="5"/>
+        <v>104.65022612023949</v>
+      </c>
+      <c r="H26" s="8">
+        <f t="shared" ref="H26" si="12">F26/20</f>
+        <v>52.325113060119747</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="1">
+        <f t="shared" ref="B27:B37" si="13">B26*POWER(2,1/12)</f>
+        <v>1108.7305239074888</v>
+      </c>
+      <c r="C27" s="1">
+        <f t="shared" si="9"/>
+        <v>0.90193241589102202</v>
+      </c>
+      <c r="D27" s="1">
+        <f t="shared" si="3"/>
+        <v>0.45096620794551101</v>
+      </c>
+      <c r="E27">
+        <f t="shared" si="7"/>
+        <v>50</v>
+      </c>
+      <c r="F27" s="7">
+        <f t="shared" ref="F27:F37" si="14">1000/C27</f>
+        <v>1108.730523907489</v>
+      </c>
+      <c r="G27" s="7">
+        <f t="shared" si="5"/>
+        <v>110.8730523907489</v>
+      </c>
+      <c r="H27" s="8">
+        <f t="shared" ref="H27:H37" si="15">F27/20</f>
+        <v>55.436526195374448</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>2</v>
+      </c>
+      <c r="B28" s="1">
+        <f t="shared" si="13"/>
+        <v>1174.6590716696307</v>
+      </c>
+      <c r="C28" s="1">
+        <f t="shared" si="9"/>
+        <v>0.85131083913447769</v>
+      </c>
+      <c r="D28" s="1">
+        <f t="shared" si="3"/>
+        <v>0.42565541956723885</v>
+      </c>
+      <c r="E28">
+        <f t="shared" si="7"/>
+        <v>47</v>
+      </c>
+      <c r="F28" s="7">
+        <f t="shared" si="14"/>
+        <v>1174.6590716696307</v>
+      </c>
+      <c r="G28" s="7">
+        <f t="shared" si="5"/>
+        <v>117.46590716696308</v>
+      </c>
+      <c r="H28" s="8">
+        <f t="shared" si="15"/>
+        <v>58.732953583481539</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="1">
+        <f t="shared" si="13"/>
+        <v>1244.5079348883241</v>
+      </c>
+      <c r="C29" s="1">
+        <f t="shared" si="9"/>
+        <v>0.80353043316653094</v>
+      </c>
+      <c r="D29" s="1">
+        <f t="shared" si="3"/>
+        <v>0.40176521658326547</v>
+      </c>
+      <c r="E29">
+        <f t="shared" si="7"/>
+        <v>45</v>
+      </c>
+      <c r="F29" s="7">
+        <f t="shared" si="14"/>
+        <v>1244.5079348883241</v>
+      </c>
+      <c r="G29" s="7">
+        <f t="shared" si="5"/>
+        <v>124.45079348883242</v>
+      </c>
+      <c r="H29" s="8">
+        <f t="shared" si="15"/>
+        <v>62.225396744416209</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" s="1">
+        <f t="shared" si="13"/>
+        <v>1318.5102276514804</v>
+      </c>
+      <c r="C30" s="1">
+        <f t="shared" si="9"/>
+        <v>0.75843173532388275</v>
+      </c>
+      <c r="D30" s="1">
+        <f t="shared" si="3"/>
+        <v>0.37921586766194137</v>
+      </c>
+      <c r="E30">
+        <f t="shared" si="7"/>
+        <v>42</v>
+      </c>
+      <c r="F30" s="7">
+        <f t="shared" si="14"/>
+        <v>1318.5102276514804</v>
+      </c>
+      <c r="G30" s="7">
+        <f t="shared" si="5"/>
+        <v>131.85102276514803</v>
+      </c>
+      <c r="H30" s="8">
+        <f t="shared" si="15"/>
+        <v>65.925511382574015</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>5</v>
+      </c>
+      <c r="B31" s="1">
+        <f t="shared" si="13"/>
+        <v>1396.9129257320162</v>
+      </c>
+      <c r="C31" s="1">
+        <f t="shared" si="9"/>
+        <v>0.71586423289481393</v>
+      </c>
+      <c r="D31" s="1">
+        <f t="shared" si="3"/>
+        <v>0.35793211644740697</v>
+      </c>
+      <c r="E31">
+        <f t="shared" si="7"/>
+        <v>40</v>
+      </c>
+      <c r="F31" s="7">
+        <f t="shared" si="14"/>
+        <v>1396.9129257320162</v>
+      </c>
+      <c r="G31" s="7">
+        <f t="shared" si="5"/>
+        <v>139.69129257320162</v>
+      </c>
+      <c r="H31" s="8">
+        <f t="shared" si="15"/>
+        <v>69.845646286600811</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>6</v>
+      </c>
+      <c r="B32" s="1">
+        <f t="shared" si="13"/>
+        <v>1479.9776908465383</v>
+      </c>
+      <c r="C32" s="1">
+        <f t="shared" si="9"/>
+        <v>0.67568586079700033</v>
+      </c>
+      <c r="D32" s="1">
+        <f t="shared" si="3"/>
+        <v>0.33784293039850016</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="7"/>
+        <v>38</v>
+      </c>
+      <c r="F32" s="7">
+        <f t="shared" si="14"/>
+        <v>1479.9776908465383</v>
+      </c>
+      <c r="G32" s="7">
+        <f t="shared" si="5"/>
+        <v>147.99776908465384</v>
+      </c>
+      <c r="H32" s="8">
+        <f t="shared" si="15"/>
+        <v>73.99888454232692</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>7</v>
+      </c>
+      <c r="B33" s="1">
+        <f t="shared" si="13"/>
+        <v>1567.981743926998</v>
+      </c>
+      <c r="C33" s="1">
+        <f t="shared" si="9"/>
+        <v>0.63776252744850703</v>
+      </c>
+      <c r="D33" s="1">
+        <f t="shared" si="3"/>
+        <v>0.31888126372425352</v>
+      </c>
+      <c r="E33">
+        <f t="shared" si="7"/>
+        <v>35</v>
+      </c>
+      <c r="F33" s="7">
+        <f t="shared" si="14"/>
+        <v>1567.981743926998</v>
+      </c>
+      <c r="G33" s="7">
+        <f t="shared" si="5"/>
+        <v>156.79817439269979</v>
+      </c>
+      <c r="H33" s="8">
+        <f t="shared" si="15"/>
+        <v>78.399087196349896</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>8</v>
+      </c>
+      <c r="B34" s="1">
+        <f t="shared" si="13"/>
+        <v>1661.2187903197814</v>
+      </c>
+      <c r="C34" s="1">
+        <f t="shared" si="9"/>
+        <v>0.60196766724959927</v>
+      </c>
+      <c r="D34" s="1">
+        <f t="shared" si="3"/>
+        <v>0.30098383362479963</v>
+      </c>
+      <c r="E34">
+        <f t="shared" si="7"/>
+        <v>33</v>
+      </c>
+      <c r="F34" s="7">
+        <f t="shared" si="14"/>
+        <v>1661.2187903197814</v>
+      </c>
+      <c r="G34" s="7">
+        <f t="shared" si="5"/>
+        <v>166.12187903197815</v>
+      </c>
+      <c r="H34" s="8">
+        <f t="shared" si="15"/>
+        <v>83.060939515989077</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>9</v>
+      </c>
+      <c r="B35" s="1">
+        <f t="shared" si="13"/>
+        <v>1760.0000000000009</v>
+      </c>
+      <c r="C35" s="1">
+        <f t="shared" si="9"/>
+        <v>0.5681818181818179</v>
+      </c>
+      <c r="D35" s="1">
+        <f t="shared" si="3"/>
+        <v>0.28409090909090895</v>
+      </c>
+      <c r="E35">
+        <f t="shared" si="7"/>
+        <v>32</v>
+      </c>
+      <c r="F35" s="7">
+        <f t="shared" si="14"/>
+        <v>1760.0000000000009</v>
+      </c>
+      <c r="G35" s="7">
+        <f t="shared" si="5"/>
+        <v>176.00000000000009</v>
+      </c>
+      <c r="H35" s="8">
+        <f t="shared" si="15"/>
+        <v>88.000000000000043</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>10</v>
+      </c>
+      <c r="B36" s="1">
+        <f t="shared" si="13"/>
+        <v>1864.6550460723606</v>
+      </c>
+      <c r="C36" s="1">
+        <f t="shared" si="9"/>
+        <v>0.53629222311459823</v>
+      </c>
+      <c r="D36" s="1">
+        <f t="shared" si="3"/>
+        <v>0.26814611155729912</v>
+      </c>
+      <c r="E36">
+        <f t="shared" si="7"/>
+        <v>30</v>
+      </c>
+      <c r="F36" s="7">
+        <f t="shared" si="14"/>
+        <v>1864.6550460723608</v>
+      </c>
+      <c r="G36" s="7">
+        <f t="shared" si="5"/>
+        <v>186.46550460723608</v>
+      </c>
+      <c r="H36" s="8">
+        <f t="shared" si="15"/>
+        <v>93.232752303618042</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>11</v>
+      </c>
+      <c r="B37" s="1">
+        <f t="shared" si="13"/>
+        <v>1975.5332050244976</v>
+      </c>
+      <c r="C37" s="1">
+        <f t="shared" si="9"/>
+        <v>0.50619245348882891</v>
+      </c>
+      <c r="D37" s="1">
+        <f t="shared" si="3"/>
+        <v>0.25309622674441445</v>
+      </c>
+      <c r="E37">
+        <f t="shared" si="7"/>
+        <v>28</v>
+      </c>
+      <c r="F37" s="7">
+        <f t="shared" si="14"/>
+        <v>1975.5332050244974</v>
+      </c>
+      <c r="G37" s="7">
+        <f t="shared" si="5"/>
+        <v>197.55332050244974</v>
+      </c>
+      <c r="H37" s="8">
+        <f t="shared" si="15"/>
+        <v>98.776660251224868</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>0</v>
+      </c>
+      <c r="B38" s="1">
+        <f t="shared" ref="B38:B49" si="16">B37*POWER(2,1/12)</f>
+        <v>2093.0045224047904</v>
+      </c>
+      <c r="C38" s="1">
+        <f t="shared" si="9"/>
+        <v>0.47778205412142843</v>
+      </c>
+      <c r="D38" s="1">
+        <f t="shared" si="3"/>
+        <v>0.23889102706071422</v>
+      </c>
+      <c r="E38">
+        <f t="shared" si="7"/>
+        <v>27</v>
+      </c>
+      <c r="F38" s="7">
+        <f t="shared" ref="F38:F49" si="17">1000/C38</f>
+        <v>2093.0045224047904</v>
+      </c>
+      <c r="G38" s="7">
+        <f t="shared" si="5"/>
+        <v>209.30045224047905</v>
+      </c>
+      <c r="H38" s="8">
+        <f t="shared" ref="H38:H49" si="18">F38/20</f>
+        <v>104.65022612023952</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>1</v>
+      </c>
+      <c r="B39" s="1">
+        <f t="shared" si="16"/>
+        <v>2217.4610478149784</v>
+      </c>
+      <c r="C39" s="1">
+        <f t="shared" si="9"/>
+        <v>0.4509662079455109</v>
+      </c>
+      <c r="D39" s="1">
+        <f t="shared" si="3"/>
+        <v>0.22548310397275545</v>
+      </c>
+      <c r="E39">
+        <f t="shared" si="7"/>
+        <v>25</v>
+      </c>
+      <c r="F39" s="7">
+        <f t="shared" si="17"/>
+        <v>2217.4610478149784</v>
+      </c>
+      <c r="G39" s="7">
+        <f t="shared" si="5"/>
+        <v>221.74610478149785</v>
+      </c>
+      <c r="H39" s="8">
+        <f t="shared" si="18"/>
+        <v>110.87305239074892</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>2</v>
+      </c>
+      <c r="B40" s="1">
+        <f t="shared" si="16"/>
+        <v>2349.3181433392624</v>
+      </c>
+      <c r="C40" s="1">
+        <f t="shared" si="9"/>
+        <v>0.42565541956723868</v>
+      </c>
+      <c r="D40" s="1">
+        <f t="shared" si="3"/>
+        <v>0.21282770978361934</v>
+      </c>
+      <c r="E40">
+        <f t="shared" si="7"/>
+        <v>24</v>
+      </c>
+      <c r="F40" s="7">
+        <f t="shared" si="17"/>
+        <v>2349.3181433392624</v>
+      </c>
+      <c r="G40" s="7">
+        <f t="shared" si="5"/>
+        <v>234.93181433392624</v>
+      </c>
+      <c r="H40" s="8">
+        <f t="shared" si="18"/>
+        <v>117.46590716696312</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>3</v>
+      </c>
+      <c r="B41" s="1">
+        <f t="shared" si="16"/>
+        <v>2489.0158697766497</v>
+      </c>
+      <c r="C41" s="1">
+        <f t="shared" si="9"/>
+        <v>0.40176521658326525</v>
+      </c>
+      <c r="D41" s="1">
+        <f t="shared" si="3"/>
+        <v>0.20088260829163262</v>
+      </c>
+      <c r="E41">
+        <f t="shared" si="7"/>
+        <v>22</v>
+      </c>
+      <c r="F41" s="7">
+        <f t="shared" si="17"/>
+        <v>2489.0158697766497</v>
+      </c>
+      <c r="G41" s="7">
+        <f t="shared" si="5"/>
+        <v>248.90158697766498</v>
+      </c>
+      <c r="H41" s="8">
+        <f t="shared" si="18"/>
+        <v>124.45079348883249</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>4</v>
+      </c>
+      <c r="B42" s="1">
+        <f t="shared" si="16"/>
+        <v>2637.0204553029621</v>
+      </c>
+      <c r="C42" s="1">
+        <f t="shared" si="9"/>
+        <v>0.37921586766194115</v>
+      </c>
+      <c r="D42" s="1">
+        <f t="shared" si="3"/>
+        <v>0.18960793383097058</v>
+      </c>
+      <c r="E42">
+        <f t="shared" si="7"/>
+        <v>21</v>
+      </c>
+      <c r="F42" s="7">
+        <f t="shared" si="17"/>
+        <v>2637.0204553029625</v>
+      </c>
+      <c r="G42" s="7">
+        <f t="shared" si="5"/>
+        <v>263.70204553029623</v>
+      </c>
+      <c r="H42" s="8">
+        <f t="shared" si="18"/>
+        <v>131.85102276514812</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>5</v>
+      </c>
+      <c r="B43" s="1">
+        <f t="shared" si="16"/>
+        <v>2793.8258514640338</v>
+      </c>
+      <c r="C43" s="1">
+        <f t="shared" si="9"/>
+        <v>0.3579321164474068</v>
+      </c>
+      <c r="D43" s="1">
+        <f t="shared" si="3"/>
+        <v>0.1789660582237034</v>
+      </c>
+      <c r="E43">
+        <f t="shared" si="7"/>
+        <v>20</v>
+      </c>
+      <c r="F43" s="7">
+        <f t="shared" si="17"/>
+        <v>2793.8258514640338</v>
+      </c>
+      <c r="G43" s="7">
+        <f t="shared" si="5"/>
+        <v>279.38258514640336</v>
+      </c>
+      <c r="H43" s="8">
+        <f t="shared" si="18"/>
+        <v>139.69129257320168</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>6</v>
+      </c>
+      <c r="B44" s="1">
+        <f t="shared" si="16"/>
+        <v>2959.9553816930784</v>
+      </c>
+      <c r="C44" s="1">
+        <f t="shared" si="9"/>
+        <v>0.33784293039849994</v>
+      </c>
+      <c r="D44" s="1">
+        <f t="shared" si="3"/>
+        <v>0.16892146519924997</v>
+      </c>
+      <c r="E44">
+        <f t="shared" si="7"/>
+        <v>19</v>
+      </c>
+      <c r="F44" s="7">
+        <f t="shared" si="17"/>
+        <v>2959.9553816930784</v>
+      </c>
+      <c r="G44" s="7">
+        <f t="shared" si="5"/>
+        <v>295.99553816930785</v>
+      </c>
+      <c r="H44" s="8">
+        <f t="shared" si="18"/>
+        <v>147.99776908465392</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>7</v>
+      </c>
+      <c r="B45" s="1">
+        <f t="shared" si="16"/>
+        <v>3135.9634878539978</v>
+      </c>
+      <c r="C45" s="1">
+        <f t="shared" si="9"/>
+        <v>0.31888126372425335</v>
+      </c>
+      <c r="D45" s="1">
+        <f t="shared" si="3"/>
+        <v>0.15944063186212667</v>
+      </c>
+      <c r="E45">
+        <f t="shared" si="7"/>
+        <v>18</v>
+      </c>
+      <c r="F45" s="7">
+        <f t="shared" si="17"/>
+        <v>3135.9634878539978</v>
+      </c>
+      <c r="G45" s="7">
+        <f t="shared" si="5"/>
+        <v>313.59634878539975</v>
+      </c>
+      <c r="H45" s="8">
+        <f t="shared" si="18"/>
+        <v>156.79817439269988</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>8</v>
+      </c>
+      <c r="B46" s="1">
+        <f t="shared" si="16"/>
+        <v>3322.4375806395647</v>
+      </c>
+      <c r="C46" s="1">
+        <f t="shared" si="9"/>
+        <v>0.30098383362479947</v>
+      </c>
+      <c r="D46" s="1">
+        <f t="shared" si="3"/>
+        <v>0.15049191681239973</v>
+      </c>
+      <c r="E46">
+        <f t="shared" si="7"/>
+        <v>17</v>
+      </c>
+      <c r="F46" s="7">
+        <f t="shared" si="17"/>
+        <v>3322.4375806395647</v>
+      </c>
+      <c r="G46" s="7">
+        <f t="shared" si="5"/>
+        <v>332.24375806395648</v>
+      </c>
+      <c r="H46" s="8">
+        <f t="shared" si="18"/>
+        <v>166.12187903197824</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>9</v>
+      </c>
+      <c r="B47" s="1">
+        <f t="shared" si="16"/>
+        <v>3520.0000000000041</v>
+      </c>
+      <c r="C47" s="1">
+        <f t="shared" si="9"/>
+        <v>0.28409090909090873</v>
+      </c>
+      <c r="D47" s="1">
+        <f t="shared" si="3"/>
+        <v>0.14204545454545436</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="7"/>
+        <v>16</v>
+      </c>
+      <c r="F47" s="7">
+        <f t="shared" si="17"/>
+        <v>3520.0000000000045</v>
+      </c>
+      <c r="G47" s="7">
+        <f t="shared" si="5"/>
+        <v>352.00000000000045</v>
+      </c>
+      <c r="H47" s="8">
+        <f t="shared" si="18"/>
+        <v>176.00000000000023</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>10</v>
+      </c>
+      <c r="B48" s="1">
+        <f t="shared" si="16"/>
+        <v>3729.310092144724</v>
+      </c>
+      <c r="C48" s="1">
+        <f t="shared" si="9"/>
+        <v>0.26814611155729895</v>
+      </c>
+      <c r="D48" s="1">
+        <f t="shared" si="3"/>
+        <v>0.13407305577864947</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="F48" s="7">
+        <f t="shared" si="17"/>
+        <v>3729.310092144724</v>
+      </c>
+      <c r="G48" s="7">
+        <f t="shared" si="5"/>
+        <v>372.9310092144724</v>
+      </c>
+      <c r="H48" s="8">
+        <f t="shared" si="18"/>
+        <v>186.4655046072362</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>11</v>
+      </c>
+      <c r="B49" s="1">
+        <f t="shared" si="16"/>
+        <v>3951.066410048998</v>
+      </c>
+      <c r="C49" s="1">
+        <f t="shared" si="9"/>
+        <v>0.25309622674441423</v>
+      </c>
+      <c r="D49" s="1">
+        <f t="shared" si="3"/>
+        <v>0.12654811337220712</v>
+      </c>
+      <c r="E49">
+        <f t="shared" si="7"/>
+        <v>14</v>
+      </c>
+      <c r="F49" s="7">
+        <f t="shared" si="17"/>
+        <v>3951.066410048998</v>
+      </c>
+      <c r="G49" s="7">
+        <f t="shared" si="5"/>
+        <v>395.10664100489981</v>
+      </c>
+      <c r="H49" s="8">
+        <f t="shared" si="18"/>
+        <v>197.55332050244991</v>
       </c>
     </row>
   </sheetData>

</xml_diff>